<commit_message>
Changes to execution plan R3 and it's subsequent tc
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/OldVishwaData.xlsx
+++ b/src/test/resources/TEST_DATA/OldVishwaData.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="inbox" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -18,7 +18,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
-    <t>inbox</t>
+    <t>subjectHeader</t>
   </si>
   <si>
     <t xml:space="preserve">RE: Reactivating Dormant Account 1003 9900 0098</t>
@@ -581,7 +581,7 @@
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>